<commit_message>
Add room number list and auto-set macro for cycling through units
- Room list (201-1605) in columns E-H with dropdown validation
- 部屋番号セット macro: cycles room numbers 3 at a time into unit blocks
- 部屋番号リセット macro: resets page counter

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EwocqYiu4GvrEA8zRoMuCM
</commit_message>
<xml_diff>
--- a/写真台帳.xlsx
+++ b/写真台帳.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,11 +27,16 @@
     </font>
     <font>
       <name val="ＭＳ Ｐゴシック"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="ＭＳ Ｐゴシック"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -43,13 +48,16 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin"/>
@@ -70,22 +78,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,251 +462,581 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A2:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.1" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.1" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="6" customHeight="1"/>
+    <row r="2" ht="20.1" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>グランドメゾン静岡ザタワー</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>号室</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20.1" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="20.1" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>あぶり試験</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>発報時表示</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20.1" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="4" ht="20.1" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>写真貼付①</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>写真貼付②</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="20.1" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>201号室</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>701号室</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>1201号室</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20.1" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>202号室</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>702号室</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>1202号室</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20.1" customHeight="1">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>203号室</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>703号室</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>1203号室</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20.1" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>204号室</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>704号室</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>1204号室</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20.1" customHeight="1">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>205号室</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>705号室</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>1205号室</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20.1" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>301号室</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>801号室</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>1301号室</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20.1" customHeight="1">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="20.1" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>302号室</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>802号室</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>1302号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="6" customHeight="1">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>303号室</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>803号室</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>1303号室</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20.1" customHeight="1">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>グランドメゾン静岡ザタワー</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>304号室</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>804号室</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>1304号室</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20.1" customHeight="1">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>あぶり試験</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>発報時表示</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>305号室</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>805号室</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>1305号室</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20.1" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>写真貼付①</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>写真貼付②</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>401号室</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>901号室</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>1401号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20.1" customHeight="1">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>402号室</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>902号室</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>1402号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20.1" customHeight="1">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>403号室</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>903号室</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>1403号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20.1" customHeight="1">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>404号室</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>904号室</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>1404号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20.1" customHeight="1">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>405号室</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>905号室</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>1405号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20.1" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>501号室</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>1001号室</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>1501号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20.1" customHeight="1">
+      <c r="A20" s="7" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>502号室</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>1002号室</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>1502号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>503号室</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>1003号室</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>1503号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20.1" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>グランドメゾン静岡ザタワー</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>号室</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20.1" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="C22" s="2" t="n"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>504号室</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>1004号室</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>1504号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20.1" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>あぶり試験</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>発報時表示</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="20.1" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>505号室</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>1005号室</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>1505号室</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20.1" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>写真貼付①</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>写真貼付②</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="20.1" customHeight="1">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-    </row>
-    <row r="18" ht="20.1" customHeight="1">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-    </row>
-    <row r="19" ht="20.1" customHeight="1">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-    </row>
-    <row r="20" ht="20.1" customHeight="1">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-    </row>
-    <row r="21" ht="20.1" customHeight="1">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-    </row>
-    <row r="22" ht="20.1" customHeight="1">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-    </row>
-    <row r="23" ht="20.1" customHeight="1">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-    </row>
-    <row r="24" ht="20.1" customHeight="1">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>601号室</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>1101号室</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>1601号室</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20.1" customHeight="1">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="n"/>
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>602号室</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>1102号室</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>1602号室</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20.1" customHeight="1">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="n"/>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>603号室</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>1103号室</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>1603号室</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20.1" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>グランドメゾン静岡ザタワー</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>号室</t>
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>604号室</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>1104号室</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>1604号室</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20.1" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>あぶり試験</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>発報時表示</t>
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>605号室</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>1105号室</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>1605号室</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20.1" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>写真貼付①</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>写真貼付②</t>
-        </is>
-      </c>
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="n"/>
     </row>
     <row r="30" ht="20.1" customHeight="1">
-      <c r="A30" s="5" t="n"/>
-      <c r="B30" s="5" t="n"/>
-    </row>
-    <row r="31" ht="20.1" customHeight="1">
-      <c r="A31" s="5" t="n"/>
-      <c r="B31" s="5" t="n"/>
-    </row>
-    <row r="32" ht="20.1" customHeight="1">
-      <c r="A32" s="5" t="n"/>
-      <c r="B32" s="5" t="n"/>
-    </row>
-    <row r="33" ht="20.1" customHeight="1">
-      <c r="A33" s="5" t="n"/>
-      <c r="B33" s="5" t="n"/>
-    </row>
-    <row r="34" ht="20.1" customHeight="1">
-      <c r="A34" s="5" t="n"/>
-      <c r="B34" s="5" t="n"/>
-    </row>
-    <row r="35" ht="20.1" customHeight="1">
-      <c r="A35" s="5" t="n"/>
-      <c r="B35" s="5" t="n"/>
-    </row>
-    <row r="36" ht="20.1" customHeight="1">
-      <c r="A36" s="5" t="n"/>
-      <c r="B36" s="5" t="n"/>
-    </row>
-    <row r="37" ht="20.1" customHeight="1">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="5" t="n"/>
-    </row>
-    <row r="38" ht="20.1" customHeight="1">
-      <c r="A38" s="5" t="n"/>
-      <c r="B38" s="5" t="n"/>
-    </row>
-    <row r="39" ht="20.1" customHeight="1">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6" t="n"/>
-    </row>
-    <row r="40" ht="10.05" customHeight="1"/>
+      <c r="A30" s="7" t="n"/>
+      <c r="B30" s="7" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A3:A13"/>
-    <mergeCell ref="A16:A26"/>
-    <mergeCell ref="B16:B26"/>
-    <mergeCell ref="B29:B39"/>
-    <mergeCell ref="B3:B13"/>
-    <mergeCell ref="A29:A39"/>
+    <mergeCell ref="A4:A10"/>
+    <mergeCell ref="A24:A30"/>
+    <mergeCell ref="B4:B10"/>
+    <mergeCell ref="A14:A20"/>
+    <mergeCell ref="B24:B30"/>
+    <mergeCell ref="B14:B20"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C2 C12 C22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="部屋番号" prompt="部屋番号を選択" type="list">
+      <formula1>'インターホン親機'!$E$4:$H$28</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9"/>
 </worksheet>

</xml_diff>